<commit_message>
(fix): stale element reference, some failed scenario, and report's screenshot in extent report
</commit_message>
<xml_diff>
--- a/data/DataUser.xlsx
+++ b/data/DataUser.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>EMAIL</t>
   </si>
@@ -49,6 +49,12 @@
   </si>
   <si>
     <t>Yy0*P1t%</t>
+  </si>
+  <si>
+    <t>digna.bins@yahoo.com</t>
+  </si>
+  <si>
+    <t>Hd9*ZCMU</t>
   </si>
 </sst>
 </file>
@@ -421,7 +427,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{290CBC4D-1AFC-4B6D-8F9B-23F8520A0F28}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="28.140625"/>
@@ -460,6 +466,14 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>